<commit_message>
Investitions-Logik bereinigt: nur DPMA + Phase-3-Hardware, Rest = Sacheinlage
BWL-Korrektur: Hardware der Gründer:innen (alte Computer/Monitore) ist
keine Investition der Gesellschaft, sondern Privatvermögen → Sacheinlage
bei UG-Umfirmierung Phase 2 (~1.000 € Zeitwert).

Echte Investitionen:
- Phase 1: 290 € DPMA-Marke (10 J AfA = 29 €/J)
- Phase 3: 6.000 € Hardware (3 neue Rechner + 3 Monitore für 4 Personen,
  3 J AfA = 2.000 €/J, finanziert aus Mikromezzanin)

Einmal-Aufwand Phase 1: 700 € (Domain/Setup + eRecht24-Templates) →
direkt in GuV. In Recht-Zeile J1 integriert (50 €/Mon laufend × 12 +
700 € einmal = 1.300 €/Jahr).

AfA-Logik: J1+J2 nur Marke 29 €/J · ab J3: 2.029 €/J (Marke + Hardware).

Updates: Excel build-script, Excel regeneriert, HTML F5 Pyramide +
Detail-Footnote, Annahmen-MD, 06-MD synchron, Sprechertext.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pitch/Finanzen/geschaeftsplan-lesekumpel.xlsx
+++ b/Pitch/Finanzen/geschaeftsplan-lesekumpel.xlsx
@@ -118,6 +118,7 @@
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,7 +127,6 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -562,114 +562,126 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Finanzierung Phase 3:</t>
+          <t>Investitionen:</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Mikromezzaninfonds II · 50.000 € · 8% p.a. · 10 J endfällig (MBG MV)</t>
+          <t>Phase 1: 290 € (DPMA-Marke). Phase 3: 6.000 € (3 neue Rechner + Monitore). Hardware Phase 1+2 = Sacheinlage (1.000 €).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Break-Even:</t>
+          <t>Finanzierung Phase 3:</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>~200 Premium (moderate Ratio: 1 Pro + 5 Kaffee pro 100 Premium → 2 Pro + 10 Kaffee/Mon.)</t>
+          <t>Mikromezzaninfonds II · 50.000 € · 8% p.a. · 10 J endfällig (MBG MV)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>Break-Even:</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>~200 Premium (moderate Ratio: 1 Pro + 5 Kaffee pro 100 Premium → 2 Pro + 10 Kaffee/Mon.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>Tragfähig (Skalierung):</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>1.700 Premium · 8.500 €/Monat Umsatz = 8.500 € Kosten</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Sheet-Struktur:</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Tab 1:</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Personal, Investitionen etc. — Übersicht 3-Jahres-Plan mit AfA</t>
-        </is>
-      </c>
+          <t>Sheet-Struktur:</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Tab 2:</t>
+          <t>Tab 1:</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Mikromezzanin — Tilgungsplan über 120 Monate</t>
+          <t>Personal, Investitionen etc. — Übersicht 3-Jahres-Plan mit AfA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Tab 3:</t>
+          <t>Tab 2:</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Liquiditätsplan — monatlich J1, dann J2-J10 (Cashflow)</t>
+          <t>Mikromezzanin — Tilgungsplan über 120 Monate</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>Tab 3:</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Liquiditätsplan — monatlich J1, dann J2-J10 (Cashflow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Tab 4:</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Rentabilitätsplan — monatlich J1, dann J2-J10 (GuV mit AfA + Zinsen)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Annahmen:</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>siehe geschaeftsplan-annahmen.md</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
+          <t>Annahmen:</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>siehe geschaeftsplan-annahmen.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
           <t>Reproduzierbar:</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>python build-geschaeftsplan.py</t>
         </is>
@@ -686,7 +698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -705,357 +717,342 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Betrag</t>
+          <t>Phase 1 (Konzeption)</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3 (Skalierung)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Rechner (2× MacBooks):</t>
+          <t>DPMA-Markenanmeldung 'Lesekumpel'</t>
         </is>
       </c>
       <c r="C2" s="5" t="n">
-        <v>4000</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Monitore/Peripherie:</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>1000</v>
+          <t>3 neue Rechner (Gründer:innen + Junior, J3)</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>5400</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Markenanmeldung DPMA:</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="n">
+          <t>3 neue Monitore (Junior + Ersatz, J3)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Summe Investitionen</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
         <v>290</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Domain/Hosting-Setup:</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Rechts-Templates (eRecht24):</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>500</v>
+      <c r="D5" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Phase 1: Eigenmittel. Phase 3: aus Mikromezzanin-Tranche (siehe Tab 2).</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>5990</v>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Finanzierung Phase 1+2: Eigenmittel (Bootstrap). Phase 3: Mikromezzanin 50.000 € (siehe Tab 2).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Sacheinlage Phase 2 (UG-Umfirmierung)</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>2 alte Rechner + 2 alte Monitore — Zeitwert, eingebracht von den Gründer:innen</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Einmal-Aufwand Phase 1 (kein Anlagegut)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>700</v>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Domain/Setup + Rechts-Templates eRecht24 — direkt in GuV, keine AfA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Kalkulatorische Abschreibung:</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Rechner</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Monitore</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Marke DPMA</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Jahre:</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>10</v>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Hardware (ab J3)</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="4" t="inlineStr">
         <is>
+          <t>Nutzungsdauer (Jahre):</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
           <t>Abschreibungsbetrag je Jahr:</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
-        <v>1333.333333333333</v>
-      </c>
-      <c r="D11" s="7" t="n">
-        <v>200</v>
-      </c>
-      <c r="E11" s="7" t="n">
+      <c r="C12" s="8" t="n">
         <v>29</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Summe AfA pro Jahr:</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>1562.333333333333</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="D12" s="8" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>AfA J1+J2 (nur Marke):</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>AfA ab J3 (Marke + Hardware):</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>2029</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Einnahmen</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Jahr 1</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Jahr 2</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Jahr 3</t>
         </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Familienpaket (Premium 4,99 €)</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>2994</v>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>17964</v>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>59880</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Pro-Accounts (14,99 €)</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>179.88</v>
-      </c>
-      <c r="D18" s="5" t="n">
-        <v>899.4</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>3597.6</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Kaffeekassen (1 €)</t>
+          <t>Familienpaket (Premium 4,99 €)</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
-        <v>36</v>
+        <v>2994</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>180</v>
+        <v>17964</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>600</v>
+        <v>59880</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="4" t="inlineStr">
         <is>
+          <t>Pro-Accounts (14,99 €)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>179.88</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>899.4</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>3597.6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Kaffeekassen (1 €)</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
           <t>Förderung (Aktion Mensch/DATIpilot)</t>
         </is>
       </c>
-      <c r="C20" s="5" t="n">
+      <c r="C22" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D20" s="5" t="n">
+      <c r="D22" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="E22" s="5" t="n">
         <v>5000</v>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="3" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Summe Einnahmen (netto)</t>
         </is>
       </c>
-      <c r="C21" s="9">
-        <f>SUM(C17:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="9">
-        <f>SUM(D17:D20)</f>
-        <v/>
-      </c>
-      <c r="E21" s="9">
-        <f>SUM(E17:E20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="C23" s="10">
+        <f>SUM(C19:C22)</f>
+        <v/>
+      </c>
+      <c r="D23" s="10">
+        <f>SUM(D19:D22)</f>
+        <v/>
+      </c>
+      <c r="E23" s="10">
+        <f>SUM(E19:E22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Ausgaben</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Jahr 1</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>Jahr 2</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>Jahr 3</t>
         </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>LLM-Token + Bildgenerierung</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>2880</v>
-      </c>
-      <c r="D25" s="5" t="n">
-        <v>17280</v>
-      </c>
-      <c r="E25" s="5" t="n">
-        <v>33600</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Stripe-Gebühren (1,4 % + 0,25 €)</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>206.93832</v>
-      </c>
-      <c r="D26" s="5" t="n">
-        <v>1226.6076</v>
-      </c>
-      <c r="E26" s="5" t="n">
-        <v>4107.0864</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Hosting · Backend · CDN</t>
+          <t>LLM-Token + Bildgenerierung</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>300</v>
+        <v>2880</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>900</v>
+        <v>17280</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>4800</v>
+        <v>33600</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Recht · Buchhaltung · Versicherung (GbR ab J1 · UG ab J2)</t>
+          <t>Stripe-Gebühren (1,4 % + 0,25 €)</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
-        <v>600</v>
+        <v>206.93832</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>3000</v>
+        <v>1226.6076</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>6000</v>
+        <v>4107.0864</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Dev-Tools · Subscriptions (Claude Max etc.)</t>
+          <t>Hosting · Backend · CDN</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
-        <v>1200</v>
+        <v>300</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>1440</v>
+        <v>900</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>1800</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Marketing · Merch · Messen</t>
+          <t>Recht · Buchhaltung · Versicherung (GbR ab J1 · UG ab J2)</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
-        <v>120</v>
+        <v>1300</v>
       </c>
       <c r="D30" s="5" t="n">
-        <v>1200</v>
+        <v>3000</v>
       </c>
       <c r="E30" s="5" t="n">
         <v>6000</v>
@@ -1064,55 +1061,55 @@
     <row r="31">
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Strom · Internet · Reisekosten · Sonstige</t>
+          <t>Dev-Tools · Subscriptions (Claude Max etc.)</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>960</v>
+        <v>1440</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>2040</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Gründer:innen-Entnahme (Teilzeit J3: 3×1.000 €)</t>
+          <t>Marketing · Merch · Messen</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>36000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Mitarbeiter:in (ab Q3 J3 für 3 Monate)</t>
+          <t>Strom · Internet · Reisekosten · Sonstige</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>0</v>
+        <v>960</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>9000</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Zinsaufwand Mikromezzanin (ab Monat 26)</t>
+          <t>Gründer:innen-Entnahme (Teilzeit J3: 3×1.000 €)</t>
         </is>
       </c>
       <c r="C34" s="5" t="n">
@@ -1122,25 +1119,57 @@
         <v>0</v>
       </c>
       <c r="E34" s="5" t="n">
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Mitarbeiter:in (ab Q3 J3 für 3 Monate)</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Zinsaufwand Mikromezzanin (ab Monat 26)</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="5" t="n">
         <v>4000</v>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="3" t="inlineStr">
+    <row r="37">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Summe Ausgaben</t>
         </is>
       </c>
-      <c r="C35" s="8">
-        <f>SUM(C25:C34)</f>
-        <v/>
-      </c>
-      <c r="D35" s="8">
-        <f>SUM(D25:D34)</f>
-        <v/>
-      </c>
-      <c r="E35" s="8">
-        <f>SUM(E25:E34)</f>
+      <c r="C37" s="9">
+        <f>SUM(C27:C36)</f>
+        <v/>
+      </c>
+      <c r="D37" s="9">
+        <f>SUM(D27:D36)</f>
+        <v/>
+      </c>
+      <c r="E37" s="9">
+        <f>SUM(E27:E36)</f>
         <v/>
       </c>
     </row>
@@ -1173,7 +1202,7 @@
           <t>Kapital:</t>
         </is>
       </c>
-      <c r="B1" s="8" t="n">
+      <c r="B1" s="9" t="n">
         <v>50000</v>
       </c>
       <c r="D1" s="3" t="inlineStr">
@@ -1181,7 +1210,7 @@
           <t>Laufzeit Monate:</t>
         </is>
       </c>
-      <c r="E1" s="10" t="n">
+      <c r="E1" s="11" t="n">
         <v>120</v>
       </c>
       <c r="G1" s="3" t="inlineStr">
@@ -1196,7 +1225,7 @@
           <t>Zinssatz p.a.:</t>
         </is>
       </c>
-      <c r="B2" s="11" t="n">
+      <c r="B2" s="12" t="n">
         <v>0.08</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -1204,7 +1233,7 @@
           <t>Monatlicher Zins:</t>
         </is>
       </c>
-      <c r="E2" s="8" t="n">
+      <c r="E2" s="9" t="n">
         <v>333.3333333333333</v>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -1214,37 +1243,37 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Monat</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Auszahlung</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>Kapital Anfang</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Zins</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>Tilgung</t>
         </is>
       </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Kapital Ende</t>
         </is>
       </c>
-      <c r="G5" s="12" t="inlineStr">
+      <c r="G5" s="13" t="inlineStr">
         <is>
           <t>Jahres-Marker</t>
         </is>
@@ -1254,15 +1283,15 @@
       <c r="A6" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="B6" s="9" t="n">
-        <v>50000</v>
-      </c>
-      <c r="C6" s="13" t="n">
+      <c r="B6" s="10" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C6" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="13" t="n"/>
-      <c r="E6" s="13" t="n"/>
-      <c r="F6" s="13" t="n">
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1270,15 +1299,15 @@
       <c r="A7" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="B7" s="13" t="n"/>
-      <c r="C7" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D7" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E7" s="13" t="n"/>
-      <c r="F7" s="13" t="n">
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1286,15 +1315,15 @@
       <c r="A8" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="B8" s="13" t="n"/>
-      <c r="C8" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D8" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E8" s="13" t="n"/>
-      <c r="F8" s="13" t="n">
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1302,15 +1331,15 @@
       <c r="A9" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="B9" s="13" t="n"/>
-      <c r="C9" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D9" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="13" t="n">
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1318,15 +1347,15 @@
       <c r="A10" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="B10" s="13" t="n"/>
-      <c r="C10" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D10" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E10" s="13" t="n"/>
-      <c r="F10" s="13" t="n">
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1334,15 +1363,15 @@
       <c r="A11" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="B11" s="13" t="n"/>
-      <c r="C11" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D11" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n">
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1350,15 +1379,15 @@
       <c r="A12" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="B12" s="13" t="n"/>
-      <c r="C12" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D12" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="13" t="n">
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1366,15 +1395,15 @@
       <c r="A13" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="B13" s="13" t="n"/>
-      <c r="C13" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D13" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="13" t="n">
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1382,15 +1411,15 @@
       <c r="A14" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="B14" s="13" t="n"/>
-      <c r="C14" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D14" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="13" t="n">
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1398,15 +1427,15 @@
       <c r="A15" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="B15" s="13" t="n"/>
-      <c r="C15" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D15" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E15" s="13" t="n"/>
-      <c r="F15" s="13" t="n">
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1414,15 +1443,15 @@
       <c r="A16" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="B16" s="13" t="n"/>
-      <c r="C16" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D16" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E16" s="13" t="n"/>
-      <c r="F16" s="13" t="n">
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1430,18 +1459,18 @@
       <c r="A17" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="B17" s="13" t="n"/>
-      <c r="C17" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D17" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E17" s="13" t="n"/>
-      <c r="F17" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
         <is>
           <t>Jahr 1</t>
         </is>
@@ -1451,15 +1480,15 @@
       <c r="A18" s="4" t="n">
         <v>37</v>
       </c>
-      <c r="B18" s="13" t="n"/>
-      <c r="C18" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D18" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="13" t="n">
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1467,15 +1496,15 @@
       <c r="A19" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="B19" s="13" t="n"/>
-      <c r="C19" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D19" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E19" s="13" t="n"/>
-      <c r="F19" s="13" t="n">
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1483,15 +1512,15 @@
       <c r="A20" s="4" t="n">
         <v>39</v>
       </c>
-      <c r="B20" s="13" t="n"/>
-      <c r="C20" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D20" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="13" t="n">
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1499,15 +1528,15 @@
       <c r="A21" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="B21" s="13" t="n"/>
-      <c r="C21" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D21" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E21" s="13" t="n"/>
-      <c r="F21" s="13" t="n">
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1515,15 +1544,15 @@
       <c r="A22" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="B22" s="13" t="n"/>
-      <c r="C22" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D22" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E22" s="13" t="n"/>
-      <c r="F22" s="13" t="n">
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1531,15 +1560,15 @@
       <c r="A23" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="B23" s="13" t="n"/>
-      <c r="C23" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D23" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="13" t="n">
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1547,15 +1576,15 @@
       <c r="A24" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="B24" s="13" t="n"/>
-      <c r="C24" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D24" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="13" t="n">
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1563,15 +1592,15 @@
       <c r="A25" s="4" t="n">
         <v>44</v>
       </c>
-      <c r="B25" s="13" t="n"/>
-      <c r="C25" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D25" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E25" s="13" t="n"/>
-      <c r="F25" s="13" t="n">
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1579,15 +1608,15 @@
       <c r="A26" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="B26" s="13" t="n"/>
-      <c r="C26" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D26" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E26" s="13" t="n"/>
-      <c r="F26" s="13" t="n">
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1595,15 +1624,15 @@
       <c r="A27" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="B27" s="13" t="n"/>
-      <c r="C27" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D27" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="13" t="n">
+      <c r="B27" s="7" t="n"/>
+      <c r="C27" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E27" s="7" t="n"/>
+      <c r="F27" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1611,15 +1640,15 @@
       <c r="A28" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="B28" s="13" t="n"/>
-      <c r="C28" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D28" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E28" s="13" t="n"/>
-      <c r="F28" s="13" t="n">
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1627,18 +1656,18 @@
       <c r="A29" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="B29" s="13" t="n"/>
-      <c r="C29" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D29" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E29" s="13" t="n"/>
-      <c r="F29" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="G29" s="10" t="inlineStr">
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G29" s="11" t="inlineStr">
         <is>
           <t>Jahr 2</t>
         </is>
@@ -1648,15 +1677,15 @@
       <c r="A30" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="B30" s="13" t="n"/>
-      <c r="C30" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D30" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E30" s="13" t="n"/>
-      <c r="F30" s="13" t="n">
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E30" s="7" t="n"/>
+      <c r="F30" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1664,15 +1693,15 @@
       <c r="A31" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="B31" s="13" t="n"/>
-      <c r="C31" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D31" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E31" s="13" t="n"/>
-      <c r="F31" s="13" t="n">
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1680,15 +1709,15 @@
       <c r="A32" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="B32" s="13" t="n"/>
-      <c r="C32" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D32" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E32" s="13" t="n"/>
-      <c r="F32" s="13" t="n">
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E32" s="7" t="n"/>
+      <c r="F32" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1696,15 +1725,15 @@
       <c r="A33" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="B33" s="13" t="n"/>
-      <c r="C33" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D33" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E33" s="13" t="n"/>
-      <c r="F33" s="13" t="n">
+      <c r="B33" s="7" t="n"/>
+      <c r="C33" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1712,15 +1741,15 @@
       <c r="A34" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="B34" s="13" t="n"/>
-      <c r="C34" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D34" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E34" s="13" t="n"/>
-      <c r="F34" s="13" t="n">
+      <c r="B34" s="7" t="n"/>
+      <c r="C34" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E34" s="7" t="n"/>
+      <c r="F34" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1728,15 +1757,15 @@
       <c r="A35" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="B35" s="13" t="n"/>
-      <c r="C35" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D35" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E35" s="13" t="n"/>
-      <c r="F35" s="13" t="n">
+      <c r="B35" s="7" t="n"/>
+      <c r="C35" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E35" s="7" t="n"/>
+      <c r="F35" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1744,15 +1773,15 @@
       <c r="A36" s="4" t="n">
         <v>55</v>
       </c>
-      <c r="B36" s="13" t="n"/>
-      <c r="C36" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D36" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E36" s="13" t="n"/>
-      <c r="F36" s="13" t="n">
+      <c r="B36" s="7" t="n"/>
+      <c r="C36" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E36" s="7" t="n"/>
+      <c r="F36" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1760,15 +1789,15 @@
       <c r="A37" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="B37" s="13" t="n"/>
-      <c r="C37" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D37" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E37" s="13" t="n"/>
-      <c r="F37" s="13" t="n">
+      <c r="B37" s="7" t="n"/>
+      <c r="C37" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E37" s="7" t="n"/>
+      <c r="F37" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1776,15 +1805,15 @@
       <c r="A38" s="4" t="n">
         <v>57</v>
       </c>
-      <c r="B38" s="13" t="n"/>
-      <c r="C38" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D38" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E38" s="13" t="n"/>
-      <c r="F38" s="13" t="n">
+      <c r="B38" s="7" t="n"/>
+      <c r="C38" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E38" s="7" t="n"/>
+      <c r="F38" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1792,15 +1821,15 @@
       <c r="A39" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="B39" s="13" t="n"/>
-      <c r="C39" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D39" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E39" s="13" t="n"/>
-      <c r="F39" s="13" t="n">
+      <c r="B39" s="7" t="n"/>
+      <c r="C39" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E39" s="7" t="n"/>
+      <c r="F39" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1808,15 +1837,15 @@
       <c r="A40" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="B40" s="13" t="n"/>
-      <c r="C40" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D40" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E40" s="13" t="n"/>
-      <c r="F40" s="13" t="n">
+      <c r="B40" s="7" t="n"/>
+      <c r="C40" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E40" s="7" t="n"/>
+      <c r="F40" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1824,18 +1853,18 @@
       <c r="A41" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="B41" s="13" t="n"/>
-      <c r="C41" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D41" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E41" s="13" t="n"/>
-      <c r="F41" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="G41" s="10" t="inlineStr">
+      <c r="B41" s="7" t="n"/>
+      <c r="C41" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E41" s="7" t="n"/>
+      <c r="F41" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
         <is>
           <t>Jahr 3</t>
         </is>
@@ -1845,15 +1874,15 @@
       <c r="A42" s="4" t="n">
         <v>61</v>
       </c>
-      <c r="B42" s="13" t="n"/>
-      <c r="C42" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D42" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E42" s="13" t="n"/>
-      <c r="F42" s="13" t="n">
+      <c r="B42" s="7" t="n"/>
+      <c r="C42" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E42" s="7" t="n"/>
+      <c r="F42" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1861,15 +1890,15 @@
       <c r="A43" s="4" t="n">
         <v>62</v>
       </c>
-      <c r="B43" s="13" t="n"/>
-      <c r="C43" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D43" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E43" s="13" t="n"/>
-      <c r="F43" s="13" t="n">
+      <c r="B43" s="7" t="n"/>
+      <c r="C43" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E43" s="7" t="n"/>
+      <c r="F43" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1877,15 +1906,15 @@
       <c r="A44" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="B44" s="13" t="n"/>
-      <c r="C44" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D44" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E44" s="13" t="n"/>
-      <c r="F44" s="13" t="n">
+      <c r="B44" s="7" t="n"/>
+      <c r="C44" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E44" s="7" t="n"/>
+      <c r="F44" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1893,15 +1922,15 @@
       <c r="A45" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="B45" s="13" t="n"/>
-      <c r="C45" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D45" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E45" s="13" t="n"/>
-      <c r="F45" s="13" t="n">
+      <c r="B45" s="7" t="n"/>
+      <c r="C45" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E45" s="7" t="n"/>
+      <c r="F45" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1909,15 +1938,15 @@
       <c r="A46" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="B46" s="13" t="n"/>
-      <c r="C46" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D46" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E46" s="13" t="n"/>
-      <c r="F46" s="13" t="n">
+      <c r="B46" s="7" t="n"/>
+      <c r="C46" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D46" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E46" s="7" t="n"/>
+      <c r="F46" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1925,15 +1954,15 @@
       <c r="A47" s="4" t="n">
         <v>66</v>
       </c>
-      <c r="B47" s="13" t="n"/>
-      <c r="C47" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D47" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E47" s="13" t="n"/>
-      <c r="F47" s="13" t="n">
+      <c r="B47" s="7" t="n"/>
+      <c r="C47" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D47" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E47" s="7" t="n"/>
+      <c r="F47" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1941,15 +1970,15 @@
       <c r="A48" s="4" t="n">
         <v>67</v>
       </c>
-      <c r="B48" s="13" t="n"/>
-      <c r="C48" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D48" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E48" s="13" t="n"/>
-      <c r="F48" s="13" t="n">
+      <c r="B48" s="7" t="n"/>
+      <c r="C48" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1957,15 +1986,15 @@
       <c r="A49" s="4" t="n">
         <v>68</v>
       </c>
-      <c r="B49" s="13" t="n"/>
-      <c r="C49" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D49" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E49" s="13" t="n"/>
-      <c r="F49" s="13" t="n">
+      <c r="B49" s="7" t="n"/>
+      <c r="C49" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D49" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E49" s="7" t="n"/>
+      <c r="F49" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1973,15 +2002,15 @@
       <c r="A50" s="4" t="n">
         <v>69</v>
       </c>
-      <c r="B50" s="13" t="n"/>
-      <c r="C50" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D50" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E50" s="13" t="n"/>
-      <c r="F50" s="13" t="n">
+      <c r="B50" s="7" t="n"/>
+      <c r="C50" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D50" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E50" s="7" t="n"/>
+      <c r="F50" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -1989,15 +2018,15 @@
       <c r="A51" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="B51" s="13" t="n"/>
-      <c r="C51" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D51" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E51" s="13" t="n"/>
-      <c r="F51" s="13" t="n">
+      <c r="B51" s="7" t="n"/>
+      <c r="C51" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D51" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E51" s="7" t="n"/>
+      <c r="F51" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2005,15 +2034,15 @@
       <c r="A52" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="B52" s="13" t="n"/>
-      <c r="C52" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D52" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E52" s="13" t="n"/>
-      <c r="F52" s="13" t="n">
+      <c r="B52" s="7" t="n"/>
+      <c r="C52" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D52" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E52" s="7" t="n"/>
+      <c r="F52" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2021,18 +2050,18 @@
       <c r="A53" s="4" t="n">
         <v>72</v>
       </c>
-      <c r="B53" s="13" t="n"/>
-      <c r="C53" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D53" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E53" s="13" t="n"/>
-      <c r="F53" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="G53" s="10" t="inlineStr">
+      <c r="B53" s="7" t="n"/>
+      <c r="C53" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D53" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E53" s="7" t="n"/>
+      <c r="F53" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G53" s="11" t="inlineStr">
         <is>
           <t>Jahr 4</t>
         </is>
@@ -2042,15 +2071,15 @@
       <c r="A54" s="4" t="n">
         <v>73</v>
       </c>
-      <c r="B54" s="13" t="n"/>
-      <c r="C54" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D54" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E54" s="13" t="n"/>
-      <c r="F54" s="13" t="n">
+      <c r="B54" s="7" t="n"/>
+      <c r="C54" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D54" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E54" s="7" t="n"/>
+      <c r="F54" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2058,15 +2087,15 @@
       <c r="A55" s="4" t="n">
         <v>74</v>
       </c>
-      <c r="B55" s="13" t="n"/>
-      <c r="C55" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D55" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E55" s="13" t="n"/>
-      <c r="F55" s="13" t="n">
+      <c r="B55" s="7" t="n"/>
+      <c r="C55" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D55" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E55" s="7" t="n"/>
+      <c r="F55" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2074,15 +2103,15 @@
       <c r="A56" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="B56" s="13" t="n"/>
-      <c r="C56" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D56" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E56" s="13" t="n"/>
-      <c r="F56" s="13" t="n">
+      <c r="B56" s="7" t="n"/>
+      <c r="C56" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D56" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E56" s="7" t="n"/>
+      <c r="F56" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2090,15 +2119,15 @@
       <c r="A57" s="4" t="n">
         <v>76</v>
       </c>
-      <c r="B57" s="13" t="n"/>
-      <c r="C57" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D57" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E57" s="13" t="n"/>
-      <c r="F57" s="13" t="n">
+      <c r="B57" s="7" t="n"/>
+      <c r="C57" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D57" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E57" s="7" t="n"/>
+      <c r="F57" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2106,15 +2135,15 @@
       <c r="A58" s="4" t="n">
         <v>77</v>
       </c>
-      <c r="B58" s="13" t="n"/>
-      <c r="C58" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D58" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E58" s="13" t="n"/>
-      <c r="F58" s="13" t="n">
+      <c r="B58" s="7" t="n"/>
+      <c r="C58" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D58" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E58" s="7" t="n"/>
+      <c r="F58" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2122,15 +2151,15 @@
       <c r="A59" s="4" t="n">
         <v>78</v>
       </c>
-      <c r="B59" s="13" t="n"/>
-      <c r="C59" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D59" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E59" s="13" t="n"/>
-      <c r="F59" s="13" t="n">
+      <c r="B59" s="7" t="n"/>
+      <c r="C59" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D59" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E59" s="7" t="n"/>
+      <c r="F59" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2138,15 +2167,15 @@
       <c r="A60" s="4" t="n">
         <v>79</v>
       </c>
-      <c r="B60" s="13" t="n"/>
-      <c r="C60" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D60" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E60" s="13" t="n"/>
-      <c r="F60" s="13" t="n">
+      <c r="B60" s="7" t="n"/>
+      <c r="C60" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D60" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E60" s="7" t="n"/>
+      <c r="F60" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2154,15 +2183,15 @@
       <c r="A61" s="4" t="n">
         <v>80</v>
       </c>
-      <c r="B61" s="13" t="n"/>
-      <c r="C61" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D61" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E61" s="13" t="n"/>
-      <c r="F61" s="13" t="n">
+      <c r="B61" s="7" t="n"/>
+      <c r="C61" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D61" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E61" s="7" t="n"/>
+      <c r="F61" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2170,15 +2199,15 @@
       <c r="A62" s="4" t="n">
         <v>81</v>
       </c>
-      <c r="B62" s="13" t="n"/>
-      <c r="C62" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D62" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E62" s="13" t="n"/>
-      <c r="F62" s="13" t="n">
+      <c r="B62" s="7" t="n"/>
+      <c r="C62" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D62" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E62" s="7" t="n"/>
+      <c r="F62" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2186,15 +2215,15 @@
       <c r="A63" s="4" t="n">
         <v>82</v>
       </c>
-      <c r="B63" s="13" t="n"/>
-      <c r="C63" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D63" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E63" s="13" t="n"/>
-      <c r="F63" s="13" t="n">
+      <c r="B63" s="7" t="n"/>
+      <c r="C63" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D63" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E63" s="7" t="n"/>
+      <c r="F63" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2202,15 +2231,15 @@
       <c r="A64" s="4" t="n">
         <v>83</v>
       </c>
-      <c r="B64" s="13" t="n"/>
-      <c r="C64" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D64" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E64" s="13" t="n"/>
-      <c r="F64" s="13" t="n">
+      <c r="B64" s="7" t="n"/>
+      <c r="C64" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E64" s="7" t="n"/>
+      <c r="F64" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2218,18 +2247,18 @@
       <c r="A65" s="4" t="n">
         <v>84</v>
       </c>
-      <c r="B65" s="13" t="n"/>
-      <c r="C65" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D65" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E65" s="13" t="n"/>
-      <c r="F65" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="G65" s="10" t="inlineStr">
+      <c r="B65" s="7" t="n"/>
+      <c r="C65" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D65" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E65" s="7" t="n"/>
+      <c r="F65" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G65" s="11" t="inlineStr">
         <is>
           <t>Jahr 5</t>
         </is>
@@ -2239,15 +2268,15 @@
       <c r="A66" s="4" t="n">
         <v>85</v>
       </c>
-      <c r="B66" s="13" t="n"/>
-      <c r="C66" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D66" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E66" s="13" t="n"/>
-      <c r="F66" s="13" t="n">
+      <c r="B66" s="7" t="n"/>
+      <c r="C66" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E66" s="7" t="n"/>
+      <c r="F66" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2255,15 +2284,15 @@
       <c r="A67" s="4" t="n">
         <v>86</v>
       </c>
-      <c r="B67" s="13" t="n"/>
-      <c r="C67" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D67" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E67" s="13" t="n"/>
-      <c r="F67" s="13" t="n">
+      <c r="B67" s="7" t="n"/>
+      <c r="C67" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D67" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E67" s="7" t="n"/>
+      <c r="F67" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2271,15 +2300,15 @@
       <c r="A68" s="4" t="n">
         <v>87</v>
       </c>
-      <c r="B68" s="13" t="n"/>
-      <c r="C68" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D68" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E68" s="13" t="n"/>
-      <c r="F68" s="13" t="n">
+      <c r="B68" s="7" t="n"/>
+      <c r="C68" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E68" s="7" t="n"/>
+      <c r="F68" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2287,15 +2316,15 @@
       <c r="A69" s="4" t="n">
         <v>88</v>
       </c>
-      <c r="B69" s="13" t="n"/>
-      <c r="C69" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D69" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E69" s="13" t="n"/>
-      <c r="F69" s="13" t="n">
+      <c r="B69" s="7" t="n"/>
+      <c r="C69" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D69" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E69" s="7" t="n"/>
+      <c r="F69" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2303,15 +2332,15 @@
       <c r="A70" s="4" t="n">
         <v>89</v>
       </c>
-      <c r="B70" s="13" t="n"/>
-      <c r="C70" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D70" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E70" s="13" t="n"/>
-      <c r="F70" s="13" t="n">
+      <c r="B70" s="7" t="n"/>
+      <c r="C70" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E70" s="7" t="n"/>
+      <c r="F70" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2319,15 +2348,15 @@
       <c r="A71" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="B71" s="13" t="n"/>
-      <c r="C71" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D71" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E71" s="13" t="n"/>
-      <c r="F71" s="13" t="n">
+      <c r="B71" s="7" t="n"/>
+      <c r="C71" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D71" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E71" s="7" t="n"/>
+      <c r="F71" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2335,15 +2364,15 @@
       <c r="A72" s="4" t="n">
         <v>91</v>
       </c>
-      <c r="B72" s="13" t="n"/>
-      <c r="C72" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D72" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E72" s="13" t="n"/>
-      <c r="F72" s="13" t="n">
+      <c r="B72" s="7" t="n"/>
+      <c r="C72" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E72" s="7" t="n"/>
+      <c r="F72" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2351,15 +2380,15 @@
       <c r="A73" s="4" t="n">
         <v>92</v>
       </c>
-      <c r="B73" s="13" t="n"/>
-      <c r="C73" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D73" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E73" s="13" t="n"/>
-      <c r="F73" s="13" t="n">
+      <c r="B73" s="7" t="n"/>
+      <c r="C73" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D73" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E73" s="7" t="n"/>
+      <c r="F73" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2367,15 +2396,15 @@
       <c r="A74" s="4" t="n">
         <v>93</v>
       </c>
-      <c r="B74" s="13" t="n"/>
-      <c r="C74" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D74" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E74" s="13" t="n"/>
-      <c r="F74" s="13" t="n">
+      <c r="B74" s="7" t="n"/>
+      <c r="C74" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E74" s="7" t="n"/>
+      <c r="F74" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2383,15 +2412,15 @@
       <c r="A75" s="4" t="n">
         <v>94</v>
       </c>
-      <c r="B75" s="13" t="n"/>
-      <c r="C75" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D75" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E75" s="13" t="n"/>
-      <c r="F75" s="13" t="n">
+      <c r="B75" s="7" t="n"/>
+      <c r="C75" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D75" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E75" s="7" t="n"/>
+      <c r="F75" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2399,15 +2428,15 @@
       <c r="A76" s="4" t="n">
         <v>95</v>
       </c>
-      <c r="B76" s="13" t="n"/>
-      <c r="C76" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D76" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E76" s="13" t="n"/>
-      <c r="F76" s="13" t="n">
+      <c r="B76" s="7" t="n"/>
+      <c r="C76" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E76" s="7" t="n"/>
+      <c r="F76" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2415,18 +2444,18 @@
       <c r="A77" s="4" t="n">
         <v>96</v>
       </c>
-      <c r="B77" s="13" t="n"/>
-      <c r="C77" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D77" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E77" s="13" t="n"/>
-      <c r="F77" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="G77" s="10" t="inlineStr">
+      <c r="B77" s="7" t="n"/>
+      <c r="C77" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D77" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E77" s="7" t="n"/>
+      <c r="F77" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G77" s="11" t="inlineStr">
         <is>
           <t>Jahr 6</t>
         </is>
@@ -2436,15 +2465,15 @@
       <c r="A78" s="4" t="n">
         <v>97</v>
       </c>
-      <c r="B78" s="13" t="n"/>
-      <c r="C78" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D78" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E78" s="13" t="n"/>
-      <c r="F78" s="13" t="n">
+      <c r="B78" s="7" t="n"/>
+      <c r="C78" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E78" s="7" t="n"/>
+      <c r="F78" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2452,15 +2481,15 @@
       <c r="A79" s="4" t="n">
         <v>98</v>
       </c>
-      <c r="B79" s="13" t="n"/>
-      <c r="C79" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D79" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E79" s="13" t="n"/>
-      <c r="F79" s="13" t="n">
+      <c r="B79" s="7" t="n"/>
+      <c r="C79" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D79" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E79" s="7" t="n"/>
+      <c r="F79" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2468,15 +2497,15 @@
       <c r="A80" s="4" t="n">
         <v>99</v>
       </c>
-      <c r="B80" s="13" t="n"/>
-      <c r="C80" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D80" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E80" s="13" t="n"/>
-      <c r="F80" s="13" t="n">
+      <c r="B80" s="7" t="n"/>
+      <c r="C80" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E80" s="7" t="n"/>
+      <c r="F80" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2484,15 +2513,15 @@
       <c r="A81" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="B81" s="13" t="n"/>
-      <c r="C81" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D81" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E81" s="13" t="n"/>
-      <c r="F81" s="13" t="n">
+      <c r="B81" s="7" t="n"/>
+      <c r="C81" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D81" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E81" s="7" t="n"/>
+      <c r="F81" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2500,15 +2529,15 @@
       <c r="A82" s="4" t="n">
         <v>101</v>
       </c>
-      <c r="B82" s="13" t="n"/>
-      <c r="C82" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D82" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E82" s="13" t="n"/>
-      <c r="F82" s="13" t="n">
+      <c r="B82" s="7" t="n"/>
+      <c r="C82" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E82" s="7" t="n"/>
+      <c r="F82" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2516,15 +2545,15 @@
       <c r="A83" s="4" t="n">
         <v>102</v>
       </c>
-      <c r="B83" s="13" t="n"/>
-      <c r="C83" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D83" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E83" s="13" t="n"/>
-      <c r="F83" s="13" t="n">
+      <c r="B83" s="7" t="n"/>
+      <c r="C83" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D83" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E83" s="7" t="n"/>
+      <c r="F83" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2532,15 +2561,15 @@
       <c r="A84" s="4" t="n">
         <v>103</v>
       </c>
-      <c r="B84" s="13" t="n"/>
-      <c r="C84" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D84" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E84" s="13" t="n"/>
-      <c r="F84" s="13" t="n">
+      <c r="B84" s="7" t="n"/>
+      <c r="C84" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D84" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E84" s="7" t="n"/>
+      <c r="F84" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2548,15 +2577,15 @@
       <c r="A85" s="4" t="n">
         <v>104</v>
       </c>
-      <c r="B85" s="13" t="n"/>
-      <c r="C85" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D85" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E85" s="13" t="n"/>
-      <c r="F85" s="13" t="n">
+      <c r="B85" s="7" t="n"/>
+      <c r="C85" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D85" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E85" s="7" t="n"/>
+      <c r="F85" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2564,15 +2593,15 @@
       <c r="A86" s="4" t="n">
         <v>105</v>
       </c>
-      <c r="B86" s="13" t="n"/>
-      <c r="C86" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D86" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E86" s="13" t="n"/>
-      <c r="F86" s="13" t="n">
+      <c r="B86" s="7" t="n"/>
+      <c r="C86" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D86" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E86" s="7" t="n"/>
+      <c r="F86" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2580,15 +2609,15 @@
       <c r="A87" s="4" t="n">
         <v>106</v>
       </c>
-      <c r="B87" s="13" t="n"/>
-      <c r="C87" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D87" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E87" s="13" t="n"/>
-      <c r="F87" s="13" t="n">
+      <c r="B87" s="7" t="n"/>
+      <c r="C87" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D87" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E87" s="7" t="n"/>
+      <c r="F87" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2596,15 +2625,15 @@
       <c r="A88" s="4" t="n">
         <v>107</v>
       </c>
-      <c r="B88" s="13" t="n"/>
-      <c r="C88" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D88" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E88" s="13" t="n"/>
-      <c r="F88" s="13" t="n">
+      <c r="B88" s="7" t="n"/>
+      <c r="C88" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D88" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E88" s="7" t="n"/>
+      <c r="F88" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2612,18 +2641,18 @@
       <c r="A89" s="4" t="n">
         <v>108</v>
       </c>
-      <c r="B89" s="13" t="n"/>
-      <c r="C89" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D89" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E89" s="13" t="n"/>
-      <c r="F89" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="G89" s="10" t="inlineStr">
+      <c r="B89" s="7" t="n"/>
+      <c r="C89" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D89" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E89" s="7" t="n"/>
+      <c r="F89" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G89" s="11" t="inlineStr">
         <is>
           <t>Jahr 7</t>
         </is>
@@ -2633,15 +2662,15 @@
       <c r="A90" s="4" t="n">
         <v>109</v>
       </c>
-      <c r="B90" s="13" t="n"/>
-      <c r="C90" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D90" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E90" s="13" t="n"/>
-      <c r="F90" s="13" t="n">
+      <c r="B90" s="7" t="n"/>
+      <c r="C90" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D90" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E90" s="7" t="n"/>
+      <c r="F90" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2649,15 +2678,15 @@
       <c r="A91" s="4" t="n">
         <v>110</v>
       </c>
-      <c r="B91" s="13" t="n"/>
-      <c r="C91" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D91" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E91" s="13" t="n"/>
-      <c r="F91" s="13" t="n">
+      <c r="B91" s="7" t="n"/>
+      <c r="C91" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D91" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E91" s="7" t="n"/>
+      <c r="F91" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2665,15 +2694,15 @@
       <c r="A92" s="4" t="n">
         <v>111</v>
       </c>
-      <c r="B92" s="13" t="n"/>
-      <c r="C92" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D92" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E92" s="13" t="n"/>
-      <c r="F92" s="13" t="n">
+      <c r="B92" s="7" t="n"/>
+      <c r="C92" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D92" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E92" s="7" t="n"/>
+      <c r="F92" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2681,15 +2710,15 @@
       <c r="A93" s="4" t="n">
         <v>112</v>
       </c>
-      <c r="B93" s="13" t="n"/>
-      <c r="C93" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D93" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E93" s="13" t="n"/>
-      <c r="F93" s="13" t="n">
+      <c r="B93" s="7" t="n"/>
+      <c r="C93" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D93" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E93" s="7" t="n"/>
+      <c r="F93" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2697,15 +2726,15 @@
       <c r="A94" s="4" t="n">
         <v>113</v>
       </c>
-      <c r="B94" s="13" t="n"/>
-      <c r="C94" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D94" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E94" s="13" t="n"/>
-      <c r="F94" s="13" t="n">
+      <c r="B94" s="7" t="n"/>
+      <c r="C94" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D94" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E94" s="7" t="n"/>
+      <c r="F94" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2713,15 +2742,15 @@
       <c r="A95" s="4" t="n">
         <v>114</v>
       </c>
-      <c r="B95" s="13" t="n"/>
-      <c r="C95" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D95" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E95" s="13" t="n"/>
-      <c r="F95" s="13" t="n">
+      <c r="B95" s="7" t="n"/>
+      <c r="C95" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D95" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E95" s="7" t="n"/>
+      <c r="F95" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2729,15 +2758,15 @@
       <c r="A96" s="4" t="n">
         <v>115</v>
       </c>
-      <c r="B96" s="13" t="n"/>
-      <c r="C96" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D96" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E96" s="13" t="n"/>
-      <c r="F96" s="13" t="n">
+      <c r="B96" s="7" t="n"/>
+      <c r="C96" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D96" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E96" s="7" t="n"/>
+      <c r="F96" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2745,15 +2774,15 @@
       <c r="A97" s="4" t="n">
         <v>116</v>
       </c>
-      <c r="B97" s="13" t="n"/>
-      <c r="C97" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D97" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E97" s="13" t="n"/>
-      <c r="F97" s="13" t="n">
+      <c r="B97" s="7" t="n"/>
+      <c r="C97" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D97" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E97" s="7" t="n"/>
+      <c r="F97" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2761,15 +2790,15 @@
       <c r="A98" s="4" t="n">
         <v>117</v>
       </c>
-      <c r="B98" s="13" t="n"/>
-      <c r="C98" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D98" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E98" s="13" t="n"/>
-      <c r="F98" s="13" t="n">
+      <c r="B98" s="7" t="n"/>
+      <c r="C98" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D98" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E98" s="7" t="n"/>
+      <c r="F98" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2777,15 +2806,15 @@
       <c r="A99" s="4" t="n">
         <v>118</v>
       </c>
-      <c r="B99" s="13" t="n"/>
-      <c r="C99" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D99" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E99" s="13" t="n"/>
-      <c r="F99" s="13" t="n">
+      <c r="B99" s="7" t="n"/>
+      <c r="C99" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D99" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E99" s="7" t="n"/>
+      <c r="F99" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2793,15 +2822,15 @@
       <c r="A100" s="4" t="n">
         <v>119</v>
       </c>
-      <c r="B100" s="13" t="n"/>
-      <c r="C100" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D100" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E100" s="13" t="n"/>
-      <c r="F100" s="13" t="n">
+      <c r="B100" s="7" t="n"/>
+      <c r="C100" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D100" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E100" s="7" t="n"/>
+      <c r="F100" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2809,18 +2838,18 @@
       <c r="A101" s="4" t="n">
         <v>120</v>
       </c>
-      <c r="B101" s="13" t="n"/>
-      <c r="C101" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D101" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E101" s="13" t="n"/>
-      <c r="F101" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="G101" s="10" t="inlineStr">
+      <c r="B101" s="7" t="n"/>
+      <c r="C101" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D101" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E101" s="7" t="n"/>
+      <c r="F101" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G101" s="11" t="inlineStr">
         <is>
           <t>Jahr 8</t>
         </is>
@@ -2830,15 +2859,15 @@
       <c r="A102" s="4" t="n">
         <v>121</v>
       </c>
-      <c r="B102" s="13" t="n"/>
-      <c r="C102" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D102" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E102" s="13" t="n"/>
-      <c r="F102" s="13" t="n">
+      <c r="B102" s="7" t="n"/>
+      <c r="C102" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D102" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E102" s="7" t="n"/>
+      <c r="F102" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2846,15 +2875,15 @@
       <c r="A103" s="4" t="n">
         <v>122</v>
       </c>
-      <c r="B103" s="13" t="n"/>
-      <c r="C103" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D103" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E103" s="13" t="n"/>
-      <c r="F103" s="13" t="n">
+      <c r="B103" s="7" t="n"/>
+      <c r="C103" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D103" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E103" s="7" t="n"/>
+      <c r="F103" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2862,15 +2891,15 @@
       <c r="A104" s="4" t="n">
         <v>123</v>
       </c>
-      <c r="B104" s="13" t="n"/>
-      <c r="C104" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D104" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E104" s="13" t="n"/>
-      <c r="F104" s="13" t="n">
+      <c r="B104" s="7" t="n"/>
+      <c r="C104" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D104" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E104" s="7" t="n"/>
+      <c r="F104" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2878,15 +2907,15 @@
       <c r="A105" s="4" t="n">
         <v>124</v>
       </c>
-      <c r="B105" s="13" t="n"/>
-      <c r="C105" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D105" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E105" s="13" t="n"/>
-      <c r="F105" s="13" t="n">
+      <c r="B105" s="7" t="n"/>
+      <c r="C105" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D105" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E105" s="7" t="n"/>
+      <c r="F105" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2894,15 +2923,15 @@
       <c r="A106" s="4" t="n">
         <v>125</v>
       </c>
-      <c r="B106" s="13" t="n"/>
-      <c r="C106" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D106" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E106" s="13" t="n"/>
-      <c r="F106" s="13" t="n">
+      <c r="B106" s="7" t="n"/>
+      <c r="C106" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D106" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E106" s="7" t="n"/>
+      <c r="F106" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2910,15 +2939,15 @@
       <c r="A107" s="4" t="n">
         <v>126</v>
       </c>
-      <c r="B107" s="13" t="n"/>
-      <c r="C107" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D107" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E107" s="13" t="n"/>
-      <c r="F107" s="13" t="n">
+      <c r="B107" s="7" t="n"/>
+      <c r="C107" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D107" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E107" s="7" t="n"/>
+      <c r="F107" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2926,15 +2955,15 @@
       <c r="A108" s="4" t="n">
         <v>127</v>
       </c>
-      <c r="B108" s="13" t="n"/>
-      <c r="C108" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D108" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E108" s="13" t="n"/>
-      <c r="F108" s="13" t="n">
+      <c r="B108" s="7" t="n"/>
+      <c r="C108" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D108" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E108" s="7" t="n"/>
+      <c r="F108" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2942,15 +2971,15 @@
       <c r="A109" s="4" t="n">
         <v>128</v>
       </c>
-      <c r="B109" s="13" t="n"/>
-      <c r="C109" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D109" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E109" s="13" t="n"/>
-      <c r="F109" s="13" t="n">
+      <c r="B109" s="7" t="n"/>
+      <c r="C109" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D109" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E109" s="7" t="n"/>
+      <c r="F109" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2958,15 +2987,15 @@
       <c r="A110" s="4" t="n">
         <v>129</v>
       </c>
-      <c r="B110" s="13" t="n"/>
-      <c r="C110" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D110" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E110" s="13" t="n"/>
-      <c r="F110" s="13" t="n">
+      <c r="B110" s="7" t="n"/>
+      <c r="C110" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D110" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E110" s="7" t="n"/>
+      <c r="F110" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2974,15 +3003,15 @@
       <c r="A111" s="4" t="n">
         <v>130</v>
       </c>
-      <c r="B111" s="13" t="n"/>
-      <c r="C111" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D111" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E111" s="13" t="n"/>
-      <c r="F111" s="13" t="n">
+      <c r="B111" s="7" t="n"/>
+      <c r="C111" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D111" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E111" s="7" t="n"/>
+      <c r="F111" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -2990,15 +3019,15 @@
       <c r="A112" s="4" t="n">
         <v>131</v>
       </c>
-      <c r="B112" s="13" t="n"/>
-      <c r="C112" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D112" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E112" s="13" t="n"/>
-      <c r="F112" s="13" t="n">
+      <c r="B112" s="7" t="n"/>
+      <c r="C112" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D112" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E112" s="7" t="n"/>
+      <c r="F112" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3006,18 +3035,18 @@
       <c r="A113" s="4" t="n">
         <v>132</v>
       </c>
-      <c r="B113" s="13" t="n"/>
-      <c r="C113" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D113" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E113" s="13" t="n"/>
-      <c r="F113" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="G113" s="10" t="inlineStr">
+      <c r="B113" s="7" t="n"/>
+      <c r="C113" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D113" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E113" s="7" t="n"/>
+      <c r="F113" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G113" s="11" t="inlineStr">
         <is>
           <t>Jahr 9</t>
         </is>
@@ -3027,15 +3056,15 @@
       <c r="A114" s="4" t="n">
         <v>133</v>
       </c>
-      <c r="B114" s="13" t="n"/>
-      <c r="C114" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D114" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E114" s="13" t="n"/>
-      <c r="F114" s="13" t="n">
+      <c r="B114" s="7" t="n"/>
+      <c r="C114" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D114" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E114" s="7" t="n"/>
+      <c r="F114" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3043,15 +3072,15 @@
       <c r="A115" s="4" t="n">
         <v>134</v>
       </c>
-      <c r="B115" s="13" t="n"/>
-      <c r="C115" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D115" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E115" s="13" t="n"/>
-      <c r="F115" s="13" t="n">
+      <c r="B115" s="7" t="n"/>
+      <c r="C115" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D115" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E115" s="7" t="n"/>
+      <c r="F115" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3059,15 +3088,15 @@
       <c r="A116" s="4" t="n">
         <v>135</v>
       </c>
-      <c r="B116" s="13" t="n"/>
-      <c r="C116" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D116" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E116" s="13" t="n"/>
-      <c r="F116" s="13" t="n">
+      <c r="B116" s="7" t="n"/>
+      <c r="C116" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D116" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E116" s="7" t="n"/>
+      <c r="F116" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3075,15 +3104,15 @@
       <c r="A117" s="4" t="n">
         <v>136</v>
       </c>
-      <c r="B117" s="13" t="n"/>
-      <c r="C117" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D117" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E117" s="13" t="n"/>
-      <c r="F117" s="13" t="n">
+      <c r="B117" s="7" t="n"/>
+      <c r="C117" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D117" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E117" s="7" t="n"/>
+      <c r="F117" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3091,15 +3120,15 @@
       <c r="A118" s="4" t="n">
         <v>137</v>
       </c>
-      <c r="B118" s="13" t="n"/>
-      <c r="C118" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D118" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E118" s="13" t="n"/>
-      <c r="F118" s="13" t="n">
+      <c r="B118" s="7" t="n"/>
+      <c r="C118" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D118" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E118" s="7" t="n"/>
+      <c r="F118" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3107,15 +3136,15 @@
       <c r="A119" s="4" t="n">
         <v>138</v>
       </c>
-      <c r="B119" s="13" t="n"/>
-      <c r="C119" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D119" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E119" s="13" t="n"/>
-      <c r="F119" s="13" t="n">
+      <c r="B119" s="7" t="n"/>
+      <c r="C119" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D119" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E119" s="7" t="n"/>
+      <c r="F119" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3123,15 +3152,15 @@
       <c r="A120" s="4" t="n">
         <v>139</v>
       </c>
-      <c r="B120" s="13" t="n"/>
-      <c r="C120" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D120" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E120" s="13" t="n"/>
-      <c r="F120" s="13" t="n">
+      <c r="B120" s="7" t="n"/>
+      <c r="C120" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D120" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E120" s="7" t="n"/>
+      <c r="F120" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3139,15 +3168,15 @@
       <c r="A121" s="4" t="n">
         <v>140</v>
       </c>
-      <c r="B121" s="13" t="n"/>
-      <c r="C121" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D121" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E121" s="13" t="n"/>
-      <c r="F121" s="13" t="n">
+      <c r="B121" s="7" t="n"/>
+      <c r="C121" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D121" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E121" s="7" t="n"/>
+      <c r="F121" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3155,15 +3184,15 @@
       <c r="A122" s="4" t="n">
         <v>141</v>
       </c>
-      <c r="B122" s="13" t="n"/>
-      <c r="C122" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D122" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E122" s="13" t="n"/>
-      <c r="F122" s="13" t="n">
+      <c r="B122" s="7" t="n"/>
+      <c r="C122" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D122" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E122" s="7" t="n"/>
+      <c r="F122" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3171,15 +3200,15 @@
       <c r="A123" s="4" t="n">
         <v>142</v>
       </c>
-      <c r="B123" s="13" t="n"/>
-      <c r="C123" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D123" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E123" s="13" t="n"/>
-      <c r="F123" s="13" t="n">
+      <c r="B123" s="7" t="n"/>
+      <c r="C123" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D123" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E123" s="7" t="n"/>
+      <c r="F123" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3187,15 +3216,15 @@
       <c r="A124" s="4" t="n">
         <v>143</v>
       </c>
-      <c r="B124" s="13" t="n"/>
-      <c r="C124" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D124" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E124" s="13" t="n"/>
-      <c r="F124" s="13" t="n">
+      <c r="B124" s="7" t="n"/>
+      <c r="C124" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D124" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E124" s="7" t="n"/>
+      <c r="F124" s="7" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3203,20 +3232,20 @@
       <c r="A125" s="4" t="n">
         <v>144</v>
       </c>
-      <c r="B125" s="13" t="n"/>
-      <c r="C125" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D125" s="13" t="n">
-        <v>333.3333333333333</v>
-      </c>
-      <c r="E125" s="8" t="n">
-        <v>50000</v>
-      </c>
-      <c r="F125" s="13" t="n">
+      <c r="B125" s="7" t="n"/>
+      <c r="C125" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D125" s="7" t="n">
+        <v>333.3333333333333</v>
+      </c>
+      <c r="E125" s="9" t="n">
+        <v>50000</v>
+      </c>
+      <c r="F125" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G125" s="10" t="inlineStr">
+      <c r="G125" s="11" t="inlineStr">
         <is>
           <t>Jahr 10</t>
         </is>
@@ -3226,13 +3255,13 @@
       <c r="A126" s="4" t="n">
         <v>145</v>
       </c>
-      <c r="B126" s="13" t="n"/>
-      <c r="C126" s="13" t="n">
+      <c r="B126" s="7" t="n"/>
+      <c r="C126" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D126" s="13" t="n"/>
-      <c r="E126" s="13" t="n"/>
-      <c r="F126" s="13" t="n">
+      <c r="D126" s="7" t="n"/>
+      <c r="E126" s="7" t="n"/>
+      <c r="F126" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3289,112 +3318,112 @@
           <t>Posten</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>Monat 1</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>Monat 2</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="D2" s="13" t="inlineStr">
         <is>
           <t>Monat 3</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="E2" s="13" t="inlineStr">
         <is>
           <t>Monat 4</t>
         </is>
       </c>
-      <c r="F2" s="12" t="inlineStr">
+      <c r="F2" s="13" t="inlineStr">
         <is>
           <t>Monat 5</t>
         </is>
       </c>
-      <c r="G2" s="12" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>Monat 6</t>
         </is>
       </c>
-      <c r="H2" s="12" t="inlineStr">
+      <c r="H2" s="13" t="inlineStr">
         <is>
           <t>Monat 7</t>
         </is>
       </c>
-      <c r="I2" s="12" t="inlineStr">
+      <c r="I2" s="13" t="inlineStr">
         <is>
           <t>Monat 8</t>
         </is>
       </c>
-      <c r="J2" s="12" t="inlineStr">
+      <c r="J2" s="13" t="inlineStr">
         <is>
           <t>Monat 9</t>
         </is>
       </c>
-      <c r="K2" s="12" t="inlineStr">
+      <c r="K2" s="13" t="inlineStr">
         <is>
           <t>Monat 10</t>
         </is>
       </c>
-      <c r="L2" s="12" t="inlineStr">
+      <c r="L2" s="13" t="inlineStr">
         <is>
           <t>Monat 11</t>
         </is>
       </c>
-      <c r="M2" s="12" t="inlineStr">
+      <c r="M2" s="13" t="inlineStr">
         <is>
           <t>Monat 12</t>
         </is>
       </c>
-      <c r="N2" s="12" t="inlineStr">
+      <c r="N2" s="13" t="inlineStr">
         <is>
           <t>Jahr 2</t>
         </is>
       </c>
-      <c r="O2" s="12" t="inlineStr">
+      <c r="O2" s="13" t="inlineStr">
         <is>
           <t>Jahr 3</t>
         </is>
       </c>
-      <c r="P2" s="12" t="inlineStr">
+      <c r="P2" s="13" t="inlineStr">
         <is>
           <t>Jahr 4</t>
         </is>
       </c>
-      <c r="Q2" s="12" t="inlineStr">
+      <c r="Q2" s="13" t="inlineStr">
         <is>
           <t>Jahr 5</t>
         </is>
       </c>
-      <c r="R2" s="12" t="inlineStr">
+      <c r="R2" s="13" t="inlineStr">
         <is>
           <t>Jahr 6</t>
         </is>
       </c>
-      <c r="S2" s="12" t="inlineStr">
+      <c r="S2" s="13" t="inlineStr">
         <is>
           <t>Jahr 7</t>
         </is>
       </c>
-      <c r="T2" s="12" t="inlineStr">
+      <c r="T2" s="13" t="inlineStr">
         <is>
           <t>Jahr 8</t>
         </is>
       </c>
-      <c r="U2" s="12" t="inlineStr">
+      <c r="U2" s="13" t="inlineStr">
         <is>
           <t>Jahr 9</t>
         </is>
       </c>
-      <c r="V2" s="12" t="inlineStr">
+      <c r="V2" s="13" t="inlineStr">
         <is>
           <t>Jahr 10</t>
         </is>
       </c>
-      <c r="W2" s="12" t="inlineStr">
+      <c r="W2" s="13" t="inlineStr">
         <is>
           <t>Summe 10J</t>
         </is>
@@ -3774,7 +3803,7 @@
       <c r="V9" s="18" t="n">
         <v>111152.4</v>
       </c>
-      <c r="W9" s="9">
+      <c r="W9" s="10">
         <f>SUM(B9:V9)</f>
         <v/>
       </c>
@@ -3793,14 +3822,10 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>490</v>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>500</v>
-      </c>
+        <v>990</v>
+      </c>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
@@ -3811,7 +3836,9 @@
       <c r="L12" s="5" t="n"/>
       <c r="M12" s="5" t="n"/>
       <c r="N12" s="5" t="n"/>
-      <c r="O12" s="5" t="n"/>
+      <c r="O12" s="5" t="n">
+        <v>6000</v>
+      </c>
       <c r="P12" s="5" t="n"/>
       <c r="Q12" s="5" t="n"/>
       <c r="R12" s="5" t="n"/>
@@ -4471,19 +4498,19 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Summe Ausgaben</t>
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>5275.958879999999</v>
+        <v>1265.95888</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>812.3016200000001</v>
+        <v>322.30162</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>863.72036</v>
+        <v>363.72036</v>
       </c>
       <c r="E23" s="6" t="n">
         <v>404.94324</v>
@@ -4516,7 +4543,7 @@
         <v>26006.6076</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>107013.7530666667</v>
+        <v>113013.7530666667</v>
       </c>
       <c r="P23" s="6" t="n">
         <v>184464.1336</v>
@@ -4539,7 +4566,7 @@
       <c r="V23" s="6" t="n">
         <v>184464.1336</v>
       </c>
-      <c r="W23" s="8">
+      <c r="W23" s="9">
         <f>SUM(B23:V23)</f>
         <v/>
       </c>
@@ -4787,112 +4814,112 @@
           <t>Posten</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>Monat 1</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>Monat 2</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="D2" s="13" t="inlineStr">
         <is>
           <t>Monat 3</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="E2" s="13" t="inlineStr">
         <is>
           <t>Monat 4</t>
         </is>
       </c>
-      <c r="F2" s="12" t="inlineStr">
+      <c r="F2" s="13" t="inlineStr">
         <is>
           <t>Monat 5</t>
         </is>
       </c>
-      <c r="G2" s="12" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>Monat 6</t>
         </is>
       </c>
-      <c r="H2" s="12" t="inlineStr">
+      <c r="H2" s="13" t="inlineStr">
         <is>
           <t>Monat 7</t>
         </is>
       </c>
-      <c r="I2" s="12" t="inlineStr">
+      <c r="I2" s="13" t="inlineStr">
         <is>
           <t>Monat 8</t>
         </is>
       </c>
-      <c r="J2" s="12" t="inlineStr">
+      <c r="J2" s="13" t="inlineStr">
         <is>
           <t>Monat 9</t>
         </is>
       </c>
-      <c r="K2" s="12" t="inlineStr">
+      <c r="K2" s="13" t="inlineStr">
         <is>
           <t>Monat 10</t>
         </is>
       </c>
-      <c r="L2" s="12" t="inlineStr">
+      <c r="L2" s="13" t="inlineStr">
         <is>
           <t>Monat 11</t>
         </is>
       </c>
-      <c r="M2" s="12" t="inlineStr">
+      <c r="M2" s="13" t="inlineStr">
         <is>
           <t>Monat 12</t>
         </is>
       </c>
-      <c r="N2" s="12" t="inlineStr">
+      <c r="N2" s="13" t="inlineStr">
         <is>
           <t>Jahr 2</t>
         </is>
       </c>
-      <c r="O2" s="12" t="inlineStr">
+      <c r="O2" s="13" t="inlineStr">
         <is>
           <t>Jahr 3</t>
         </is>
       </c>
-      <c r="P2" s="12" t="inlineStr">
+      <c r="P2" s="13" t="inlineStr">
         <is>
           <t>Jahr 4</t>
         </is>
       </c>
-      <c r="Q2" s="12" t="inlineStr">
+      <c r="Q2" s="13" t="inlineStr">
         <is>
           <t>Jahr 5</t>
         </is>
       </c>
-      <c r="R2" s="12" t="inlineStr">
+      <c r="R2" s="13" t="inlineStr">
         <is>
           <t>Jahr 6</t>
         </is>
       </c>
-      <c r="S2" s="12" t="inlineStr">
+      <c r="S2" s="13" t="inlineStr">
         <is>
           <t>Jahr 7</t>
         </is>
       </c>
-      <c r="T2" s="12" t="inlineStr">
+      <c r="T2" s="13" t="inlineStr">
         <is>
           <t>Jahr 8</t>
         </is>
       </c>
-      <c r="U2" s="12" t="inlineStr">
+      <c r="U2" s="13" t="inlineStr">
         <is>
           <t>Jahr 9</t>
         </is>
       </c>
-      <c r="V2" s="12" t="inlineStr">
+      <c r="V2" s="13" t="inlineStr">
         <is>
           <t>Jahr 10</t>
         </is>
       </c>
-      <c r="W2" s="12" t="inlineStr">
+      <c r="W2" s="13" t="inlineStr">
         <is>
           <t>Summe 10J</t>
         </is>
@@ -5238,7 +5265,7 @@
       <c r="V8" s="18" t="n">
         <v>111152.4</v>
       </c>
-      <c r="W8" s="9">
+      <c r="W8" s="10">
         <f>SUM(B8:V8)</f>
         <v/>
       </c>
@@ -5823,52 +5850,52 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>130.1944444444444</v>
+        <v>2.416666666666667</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>130.1944444444444</v>
+        <v>2.416666666666667</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>130.1944444444444</v>
+        <v>2.416666666666667</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>130.1944444444444</v>
+        <v>2.416666666666667</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>130.1944444444444</v>
+        <v>2.416666666666667</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>130.1944444444444</v>
+        <v>2.416666666666667</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>130.1944444444444</v>
+        <v>2.416666666666667</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>130.1944444444444</v>
+        <v>2.416666666666667</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>130.1944444444444</v>
+        <v>2.416666666666667</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>130.1944444444444</v>
+        <v>2.416666666666667</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>130.1944444444444</v>
+        <v>2.416666666666667</v>
       </c>
       <c r="M19" s="5" t="n">
-        <v>130.1944444444444</v>
+        <v>2.416666666666667</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>1562.333333333333</v>
+        <v>29</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>1562.333333333333</v>
+        <v>2029</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>229</v>
+        <v>2029</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>229</v>
+        <v>2029</v>
       </c>
       <c r="R19" s="5" t="n">
         <v>29</v>
@@ -5939,58 +5966,58 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Summe Aufwendungen</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>376.1533244444444</v>
+        <v>248.3755466666667</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>422.4960644444444</v>
+        <v>294.7182866666667</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>463.9148044444445</v>
+        <v>336.1370266666667</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>505.1376844444445</v>
+        <v>377.3599066666667</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>551.2164244444444</v>
+        <v>423.4386466666667</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>592.6351644444444</v>
+        <v>464.8573866666667</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>633.8580444444444</v>
+        <v>506.0802666666667</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>679.9367844444445</v>
+        <v>552.1590066666666</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>721.1596644444445</v>
+        <v>593.3818866666667</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>762.1185444444444</v>
+        <v>634.3407666666667</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>808.9211444444444</v>
+        <v>681.1433666666667</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>849.8800244444444</v>
+        <v>722.1022466666667</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>27568.94093333333</v>
+        <v>26035.6076</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>108576.0864</v>
+        <v>109042.7530666667</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>184693.1336</v>
+        <v>186493.1336</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>184693.1336</v>
+        <v>186493.1336</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>184493.1336</v>
@@ -6007,7 +6034,7 @@
       <c r="V21" s="6" t="n">
         <v>184493.1336</v>
       </c>
-      <c r="W21" s="8">
+      <c r="W21" s="9">
         <f>SUM(B21:V21)</f>
         <v/>
       </c>

</xml_diff>